<commit_message>
Updated toxicity, PCA, rel freq plots for publication
</commit_message>
<xml_diff>
--- a/Zinc/5. Cluster analysis/Clustering by sample results/PCA_loadings.xlsx
+++ b/Zinc/5. Cluster analysis/Clustering by sample results/PCA_loadings.xlsx
@@ -23,40 +23,40 @@
     <t xml:space="preserve">PC2</t>
   </si>
   <si>
-    <t xml:space="preserve">Temp</t>
+    <t xml:space="preserve">log_Temp_C</t>
   </si>
   <si>
     <t xml:space="preserve">pH</t>
   </si>
   <si>
-    <t xml:space="preserve">DOC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cl-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SO4 2-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cu</t>
+    <t xml:space="preserve">log_DOC_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_DIC_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Cl_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Ca_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Mg_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_SO4_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Na_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_K_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Zn_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Cu_uM</t>
   </si>
 </sst>
 </file>

</xml_diff>